<commit_message>
Live-schemasida + automatisk uppdatering via cupmanager-API och GitHub Actions
- fetch_matches.py: hämtar matcher från cupmanagers publika API, filtrerar på
  de 6 lagens id, skriver matches.json (bara vid ändring). Plockar upp
  slutspelsmatcher automatiskt.
- schedule.py: gemensam laddare (matches.json -> annars statisk seed).
- build_site.py: ny live-schemasida (filter, nu/härnäst, nedräkning) + PWA-manifest.
- build_ics.py/build_excel.py: använder gemensam laddare; SEQUENCE drivs av ändringstid.
- .github/workflows/update.yml: cron var 30:e min + manuell körning, committar vid ändring.
</commit_message>
<xml_diff>
--- a/Alingsas_HK_Ahus_Beach_2026.xlsx
+++ b/Alingsas_HK_Ahus_Beach_2026.xlsx
@@ -90,12 +90,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007A7A7A"/>
+        <fgColor rgb="002E5C8A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E5C8A"/>
+        <fgColor rgb="007A7A7A"/>
       </patternFill>
     </fill>
     <fill>
@@ -767,11 +767,11 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>P15 Vit</t>
+          <t>P15 Blå</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -781,27 +781,27 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK VIT</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>IFK Malmö HF</t>
+          <t>Grupp 2</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Lugi HF 3</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>IFK Malmö HF</t>
+          <t>Lugi HF 3</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -822,11 +822,11 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>P15 Blå</t>
+          <t>P15 Vit</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -836,27 +836,27 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>Lugi HF 3</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Blå</t>
+          <t>Grupp 1</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK VIT</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>IFK Malmö HF</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Lugi HF 3</t>
+          <t>IFK Malmö HF</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -1097,11 +1097,11 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>P15 Vit</t>
+          <t>P15 Blå</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1111,22 +1111,22 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
+          <t>Grupp 2</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>IFK Tumba HK 2</t>
+          <t>Staffanstorps HK</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK VIT</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>IFK Tumba HK 2</t>
+          <t>Staffanstorps HK</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
@@ -1152,11 +1152,11 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>P15 Blå</t>
+          <t>P15 Vit</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1166,22 +1166,22 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
+          <t>Grupp 1</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Staffanstorps HK</t>
+          <t>IFK Tumba HK 2</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Blå</t>
+          <t>Alingsås HK VIT</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>Staffanstorps HK</t>
+          <t>IFK Tumba HK 2</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -1317,11 +1317,11 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>F15 Gul</t>
+        <v>11</v>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>F15 Vit</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1331,27 +1331,27 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Grupp 3</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Gul</t>
-        </is>
-      </c>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>H43 Lund HF 2</t>
+          <t>Grupp 4</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Gustavsbergs IF HK</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Vit</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>H43 Lund HF 2</t>
+          <t>Gustavsbergs IF HK</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -1372,11 +1372,11 @@
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>F15 Vit</t>
+        <v>8</v>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>F15 Gul</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1386,27 +1386,27 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>Gustavsbergs IF HK</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Vit</t>
+          <t>Grupp 3</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Gul</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>H43 Lund HF 2</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>Gustavsbergs IF HK</t>
+          <t>H43 Lund HF 2</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       <c r="D20" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>P15 Vit</t>
         </is>
@@ -1484,7 +1484,7 @@
       <c r="D21" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>P15 Blå</t>
         </is>
@@ -1759,7 +1759,7 @@
       <c r="D26" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>P15 Vit</t>
         </is>
@@ -1814,7 +1814,7 @@
       <c r="D27" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>P15 Blå</t>
         </is>
@@ -2034,7 +2034,7 @@
       <c r="D31" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>P15 Vit</t>
         </is>
@@ -2087,11 +2087,11 @@
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>P15 Blå</t>
+        <v>14</v>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>P15 Orange</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -2101,22 +2101,22 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
+          <t>Grupp 4</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Blå</t>
+          <t>Alingsås HK Orange</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>Ystads IF HF</t>
+          <t>Lugi HF 4</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Ystads IF HF</t>
+          <t>Lugi HF 4</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
@@ -2142,11 +2142,11 @@
         </is>
       </c>
       <c r="D33" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="E33" s="11" t="inlineStr">
-        <is>
-          <t>P15 Orange</t>
+        <v>2</v>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>P15 Blå</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2156,22 +2156,22 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
+          <t>Grupp 2</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Orange</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>Lugi HF 4</t>
+          <t>Ystads IF HF</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Lugi HF 4</t>
+          <t>Ystads IF HF</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
@@ -2362,11 +2362,11 @@
         </is>
       </c>
       <c r="D37" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>P15 Vit</t>
+        <v>15</v>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>P15 Orange</t>
         </is>
       </c>
       <c r="F37" s="13" t="inlineStr">
@@ -2376,27 +2376,27 @@
       </c>
       <c r="G37" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
-        </is>
-      </c>
-      <c r="H37" s="14" t="inlineStr">
-        <is>
-          <t>Höörs HK H 65 vit</t>
-        </is>
-      </c>
-      <c r="I37" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK VIT</t>
+          <t>Grupp 4</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Orange</t>
+        </is>
+      </c>
+      <c r="I37" s="14" t="inlineStr">
+        <is>
+          <t>Täby HBK</t>
         </is>
       </c>
       <c r="J37" s="14" t="inlineStr">
         <is>
-          <t>Höörs HK H 65 vit</t>
+          <t>Täby HBK</t>
         </is>
       </c>
       <c r="K37" s="13" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -2417,11 +2417,11 @@
         </is>
       </c>
       <c r="D38" s="13" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
-          <t>P15 Blå</t>
+          <t>P15 Vit</t>
         </is>
       </c>
       <c r="F38" s="13" t="inlineStr">
@@ -2431,27 +2431,27 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Blå</t>
-        </is>
-      </c>
-      <c r="I38" s="14" t="inlineStr">
-        <is>
-          <t>H43 Lund HF 2</t>
+          <t>Grupp 1</t>
+        </is>
+      </c>
+      <c r="H38" s="14" t="inlineStr">
+        <is>
+          <t>Höörs HK H 65 H65 vit</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK VIT</t>
         </is>
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>H43 Lund HF 2</t>
+          <t>Höörs HK H 65 H65 vit</t>
         </is>
       </c>
       <c r="K38" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -2472,11 +2472,11 @@
         </is>
       </c>
       <c r="D39" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="E39" s="11" t="inlineStr">
-        <is>
-          <t>P15 Orange</t>
+        <v>7</v>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>P15 Blå</t>
         </is>
       </c>
       <c r="F39" s="13" t="inlineStr">
@@ -2486,22 +2486,22 @@
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
+          <t>Grupp 2</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Orange</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="I39" s="14" t="inlineStr">
         <is>
-          <t>Täby HBK</t>
+          <t>H43 Lund HF 2</t>
         </is>
       </c>
       <c r="J39" s="14" t="inlineStr">
         <is>
-          <t>Täby HBK</t>
+          <t>H43 Lund HF 2</t>
         </is>
       </c>
       <c r="K39" s="13" t="inlineStr">
@@ -2637,11 +2637,11 @@
         </is>
       </c>
       <c r="D42" s="13" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>P15 Vit</t>
+          <t>P15 Blå</t>
         </is>
       </c>
       <c r="F42" s="13" t="inlineStr">
@@ -2651,22 +2651,22 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
+          <t>Grupp 2</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK VIT</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="I42" s="14" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 3</t>
+          <t>Malmslätts HF</t>
         </is>
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 3</t>
+          <t>Malmslätts HF</t>
         </is>
       </c>
       <c r="K42" s="13" t="inlineStr">
@@ -2692,11 +2692,11 @@
         </is>
       </c>
       <c r="D43" s="13" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>P15 Blå</t>
+          <t>P15 Vit</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr">
@@ -2706,22 +2706,22 @@
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
+          <t>Grupp 1</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Blå</t>
+          <t>Alingsås HK VIT</t>
         </is>
       </c>
       <c r="I43" s="14" t="inlineStr">
         <is>
-          <t>Malmslätts HF</t>
+          <t>IFK Kristianstad 3</t>
         </is>
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>Malmslätts HF</t>
+          <t>IFK Kristianstad 3</t>
         </is>
       </c>
       <c r="K43" s="13" t="inlineStr">
@@ -2802,11 +2802,11 @@
         </is>
       </c>
       <c r="D45" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>F15 Blå</t>
+        <v>13</v>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>F15 Vit</t>
         </is>
       </c>
       <c r="F45" s="13" t="inlineStr">
@@ -2816,27 +2816,27 @@
       </c>
       <c r="G45" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
-        </is>
-      </c>
-      <c r="H45" s="14" t="inlineStr">
-        <is>
-          <t>Lödde Vikings HK Svart</t>
-        </is>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Blå</t>
+          <t>Grupp 4</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Vit</t>
+        </is>
+      </c>
+      <c r="I45" s="14" t="inlineStr">
+        <is>
+          <t>Ystads IF HF 1</t>
         </is>
       </c>
       <c r="J45" s="14" t="inlineStr">
         <is>
-          <t>Lödde Vikings HK Svart</t>
+          <t>Ystads IF HF 1</t>
         </is>
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -2857,11 +2857,11 @@
         </is>
       </c>
       <c r="D46" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>F15 Gul</t>
+        <v>2</v>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>F15 Blå</t>
         </is>
       </c>
       <c r="F46" s="13" t="inlineStr">
@@ -2871,22 +2871,22 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>Grupp 3</t>
+          <t>Grupp 1</t>
         </is>
       </c>
       <c r="H46" s="14" t="inlineStr">
         <is>
-          <t>Önnereds HK 1</t>
+          <t>Lödde Vikings HK Svart</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Gul</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>Önnereds HK 1</t>
+          <t>Lödde Vikings HK Svart</t>
         </is>
       </c>
       <c r="K46" s="13" t="inlineStr">
@@ -2912,11 +2912,11 @@
         </is>
       </c>
       <c r="D47" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>F15 Vit</t>
+        <v>8</v>
+      </c>
+      <c r="E47" s="12" t="inlineStr">
+        <is>
+          <t>F15 Gul</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr">
@@ -2926,27 +2926,27 @@
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Vit</t>
-        </is>
-      </c>
-      <c r="I47" s="14" t="inlineStr">
-        <is>
-          <t>Ystads IF HF 1</t>
+          <t>Grupp 3</t>
+        </is>
+      </c>
+      <c r="H47" s="14" t="inlineStr">
+        <is>
+          <t>Önnereds HK 1</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Gul</t>
         </is>
       </c>
       <c r="J47" s="14" t="inlineStr">
         <is>
-          <t>Ystads IF HF 1</t>
+          <t>Önnereds HK 1</t>
         </is>
       </c>
       <c r="K47" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -2967,11 +2967,11 @@
         </is>
       </c>
       <c r="D48" s="13" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>P15 Vit</t>
+          <t>P15 Blå</t>
         </is>
       </c>
       <c r="F48" s="13" t="inlineStr">
@@ -2981,22 +2981,22 @@
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
+          <t>Grupp 2</t>
         </is>
       </c>
       <c r="H48" s="14" t="inlineStr">
         <is>
-          <t>H43 Lund HF 1</t>
+          <t>HF Karlskrona Svart</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK VIT</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>H43 Lund HF 1</t>
+          <t>HF Karlskrona Svart</t>
         </is>
       </c>
       <c r="K48" s="13" t="inlineStr">
@@ -3022,11 +3022,11 @@
         </is>
       </c>
       <c r="D49" s="13" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>P15 Blå</t>
+          <t>P15 Vit</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr">
@@ -3036,22 +3036,22 @@
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
+          <t>Grupp 1</t>
         </is>
       </c>
       <c r="H49" s="14" t="inlineStr">
         <is>
-          <t>HF Karlskrona Svart</t>
+          <t>H43 Lund HF 1</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Blå</t>
+          <t>Alingsås HK VIT</t>
         </is>
       </c>
       <c r="J49" s="14" t="inlineStr">
         <is>
-          <t>HF Karlskrona Svart</t>
+          <t>H43 Lund HF 1</t>
         </is>
       </c>
       <c r="K49" s="13" t="inlineStr">
@@ -3132,11 +3132,11 @@
         </is>
       </c>
       <c r="D51" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>F15 Blå</t>
+        <v>13</v>
+      </c>
+      <c r="E51" s="12" t="inlineStr">
+        <is>
+          <t>F15 Gul</t>
         </is>
       </c>
       <c r="F51" s="13" t="inlineStr">
@@ -3146,27 +3146,27 @@
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Blå</t>
-        </is>
-      </c>
-      <c r="I51" s="14" t="inlineStr">
-        <is>
-          <t>Huddinge HK 1</t>
+          <t>Grupp 3</t>
+        </is>
+      </c>
+      <c r="H51" s="14" t="inlineStr">
+        <is>
+          <t>IFK Tumba HK Vit</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Gul</t>
         </is>
       </c>
       <c r="J51" s="14" t="inlineStr">
         <is>
-          <t>Huddinge HK 1</t>
+          <t>IFK Tumba HK Vit</t>
         </is>
       </c>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -3187,11 +3187,11 @@
         </is>
       </c>
       <c r="D52" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="E52" s="12" t="inlineStr">
-        <is>
-          <t>F15 Gul</t>
+        <v>17</v>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>F15 Vit</t>
         </is>
       </c>
       <c r="F52" s="13" t="inlineStr">
@@ -3201,27 +3201,27 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>Grupp 3</t>
-        </is>
-      </c>
-      <c r="H52" s="14" t="inlineStr">
-        <is>
-          <t>IFK Tumba HK Vit</t>
-        </is>
-      </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Gul</t>
+          <t>Grupp 4</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Vit</t>
+        </is>
+      </c>
+      <c r="I52" s="14" t="inlineStr">
+        <is>
+          <t>Huddinge HK 2</t>
         </is>
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>IFK Tumba HK Vit</t>
+          <t>Huddinge HK 2</t>
         </is>
       </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -3242,11 +3242,11 @@
         </is>
       </c>
       <c r="D53" s="13" t="n">
-        <v>17</v>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>F15 Vit</t>
+        <v>3</v>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>F15 Blå</t>
         </is>
       </c>
       <c r="F53" s="13" t="inlineStr">
@@ -3256,22 +3256,22 @@
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
+          <t>Grupp 1</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Vit</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="I53" s="14" t="inlineStr">
         <is>
-          <t>Huddinge HK 2</t>
+          <t>Huddinge HK 1</t>
         </is>
       </c>
       <c r="J53" s="14" t="inlineStr">
         <is>
-          <t>Huddinge HK 2</t>
+          <t>Huddinge HK 1</t>
         </is>
       </c>
       <c r="K53" s="13" t="inlineStr">
@@ -3299,7 +3299,7 @@
       <c r="D54" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="E54" s="9" t="inlineStr">
+      <c r="E54" s="10" t="inlineStr">
         <is>
           <t>P15 Vit</t>
         </is>
@@ -3354,7 +3354,7 @@
       <c r="D55" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="E55" s="10" t="inlineStr">
+      <c r="E55" s="9" t="inlineStr">
         <is>
           <t>P15 Blå</t>
         </is>
@@ -5044,7 +5044,7 @@
       </c>
       <c r="H10" s="14" t="inlineStr">
         <is>
-          <t>Höörs HK H 65 vit</t>
+          <t>Höörs HK H 65 H65 vit</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>Höörs HK H 65 vit</t>
+          <t>Höörs HK H 65 H65 vit</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Auto-uppdatering av schema (2026-07-04 14:09 UTC)
</commit_message>
<xml_diff>
--- a/Alingsas_HK_Ahus_Beach_2026.xlsx
+++ b/Alingsas_HK_Ahus_Beach_2026.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Info &amp; slutspel" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Alla matcher'!$A$5:$K$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Alla matcher'!$A$5:$K$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -846,12 +846,12 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>IFK Malmö HF</t>
+          <t>IFK Malmö HF 1</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>IFK Malmö HF</t>
+          <t>IFK Malmö HF 1</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 1</t>
+          <t>Spånga HK Vit</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 1</t>
+          <t>Spånga HK Vit</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
@@ -1554,24 +1554,24 @@
           <t>Grupp 4</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Eslövs HK Svart</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>Alingsås HK Orange</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>Spånga HK Vit</t>
-        </is>
-      </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>Spånga HK Vit</t>
+          <t>Eslövs HK Svart</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -1884,24 +1884,24 @@
           <t>Grupp 4</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>Eslövs HK Svart</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Alingsås HK Orange</t>
         </is>
       </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>Lugi HF 4</t>
+        </is>
+      </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>Eslövs HK Svart</t>
+          <t>Lugi HF 4</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
@@ -2111,12 +2111,12 @@
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>Lugi HF 4</t>
+          <t>Täby HBK</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Lugi HF 4</t>
+          <t>Täby HBK</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
@@ -2193,45 +2193,45 @@
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D34" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>F15 Blå</t>
+        <v>6</v>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>P15 Orange</t>
         </is>
       </c>
       <c r="F34" s="13" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Blå</t>
-        </is>
-      </c>
-      <c r="I34" s="14" t="inlineStr">
-        <is>
-          <t>IFK Kristianstad 2</t>
+          <t>Grupp 4</t>
+        </is>
+      </c>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t>Dalby GIF 1</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Orange</t>
         </is>
       </c>
       <c r="J34" s="14" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 2</t>
+          <t>Dalby GIF 1</t>
         </is>
       </c>
       <c r="K34" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -2248,15 +2248,15 @@
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="D35" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>F15 Gul</t>
+        <v>11</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>F15 Blå</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr">
@@ -2266,27 +2266,27 @@
       </c>
       <c r="G35" s="13" t="inlineStr">
         <is>
-          <t>Grupp 3</t>
-        </is>
-      </c>
-      <c r="H35" s="14" t="inlineStr">
-        <is>
-          <t>IFK Kristianstad 1</t>
-        </is>
-      </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Gul</t>
+          <t>Grupp 1</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Blå</t>
+        </is>
+      </c>
+      <c r="I35" s="14" t="inlineStr">
+        <is>
+          <t>IFK Kristianstad 2</t>
         </is>
       </c>
       <c r="J35" s="14" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 1</t>
+          <t>IFK Kristianstad 2</t>
         </is>
       </c>
       <c r="K35" s="13" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -2307,11 +2307,11 @@
         </is>
       </c>
       <c r="D36" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>F15 Vit</t>
+        <v>1</v>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>F15 Gul</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr">
@@ -2321,22 +2321,22 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
+          <t>Grupp 3</t>
         </is>
       </c>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>IFK Malmö HF Gul</t>
+          <t>IFK Kristianstad 1</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Vit</t>
+          <t>Alingsås HK Gul</t>
         </is>
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>IFK Malmö HF Gul</t>
+          <t>IFK Kristianstad 1</t>
         </is>
       </c>
       <c r="K36" s="13" t="inlineStr">
@@ -2358,20 +2358,20 @@
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="D37" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>P15 Orange</t>
+        <v>3</v>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>F15 Vit</t>
         </is>
       </c>
       <c r="F37" s="13" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="G37" s="13" t="inlineStr">
@@ -2379,24 +2379,24 @@
           <t>Grupp 4</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Orange</t>
-        </is>
-      </c>
-      <c r="I37" s="14" t="inlineStr">
-        <is>
-          <t>Täby HBK</t>
+      <c r="H37" s="14" t="inlineStr">
+        <is>
+          <t>IFK Malmö HF Gul</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Vit</t>
         </is>
       </c>
       <c r="J37" s="14" t="inlineStr">
         <is>
-          <t>Täby HBK</t>
+          <t>IFK Malmö HF Gul</t>
         </is>
       </c>
       <c r="K37" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -2417,11 +2417,11 @@
         </is>
       </c>
       <c r="D38" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E38" s="10" t="inlineStr">
-        <is>
-          <t>P15 Vit</t>
+        <v>16</v>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>P15 Orange</t>
         </is>
       </c>
       <c r="F38" s="13" t="inlineStr">
@@ -2431,22 +2431,22 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
+          <t>Grupp 4</t>
         </is>
       </c>
       <c r="H38" s="14" t="inlineStr">
         <is>
-          <t>Höörs HK H 65 H65 vit</t>
+          <t>IF Hallby HK Svart</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK VIT</t>
+          <t>Alingsås HK Orange</t>
         </is>
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>Höörs HK H 65 H65 vit</t>
+          <t>IF Hallby HK Svart</t>
         </is>
       </c>
       <c r="K38" s="13" t="inlineStr">
@@ -2472,11 +2472,11 @@
         </is>
       </c>
       <c r="D39" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>P15 Blå</t>
+        <v>3</v>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>P15 Vit</t>
         </is>
       </c>
       <c r="F39" s="13" t="inlineStr">
@@ -2486,27 +2486,27 @@
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Blå</t>
-        </is>
-      </c>
-      <c r="I39" s="14" t="inlineStr">
-        <is>
-          <t>H43 Lund HF 2</t>
+          <t>Grupp 1</t>
+        </is>
+      </c>
+      <c r="H39" s="14" t="inlineStr">
+        <is>
+          <t>Höörs HK H 65 H65 vit</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK VIT</t>
         </is>
       </c>
       <c r="J39" s="14" t="inlineStr">
         <is>
-          <t>H43 Lund HF 2</t>
+          <t>Höörs HK H 65 H65 vit</t>
         </is>
       </c>
       <c r="K39" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -2523,45 +2523,45 @@
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="D40" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="E40" s="12" t="inlineStr">
-        <is>
-          <t>F15 Gul</t>
+        <v>7</v>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>P15 Blå</t>
         </is>
       </c>
       <c r="F40" s="13" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t>Grupp 3</t>
-        </is>
-      </c>
-      <c r="H40" s="14" t="inlineStr">
-        <is>
-          <t>IFK Malmö HF Vit</t>
-        </is>
-      </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Gul</t>
+          <t>Grupp 2</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Blå</t>
+        </is>
+      </c>
+      <c r="I40" s="14" t="inlineStr">
+        <is>
+          <t>H43 Lund HF 2</t>
         </is>
       </c>
       <c r="J40" s="14" t="inlineStr">
         <is>
-          <t>IFK Malmö HF Vit</t>
+          <t>H43 Lund HF 2</t>
         </is>
       </c>
       <c r="K40" s="13" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -2582,11 +2582,11 @@
         </is>
       </c>
       <c r="D41" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>F15 Vit</t>
+        <v>10</v>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>F15 Gul</t>
         </is>
       </c>
       <c r="F41" s="13" t="inlineStr">
@@ -2596,27 +2596,27 @@
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Vit</t>
-        </is>
-      </c>
-      <c r="I41" s="14" t="inlineStr">
-        <is>
-          <t>Lödde Vikings HK Röd</t>
+          <t>Grupp 3</t>
+        </is>
+      </c>
+      <c r="H41" s="14" t="inlineStr">
+        <is>
+          <t>IFK Malmö HF Vit</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Gul</t>
         </is>
       </c>
       <c r="J41" s="14" t="inlineStr">
         <is>
-          <t>Lödde Vikings HK Röd</t>
+          <t>IFK Malmö HF Vit</t>
         </is>
       </c>
       <c r="K41" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -2633,40 +2633,40 @@
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="D42" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="E42" s="9" t="inlineStr">
-        <is>
-          <t>P15 Blå</t>
+        <v>13</v>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>F15 Vit</t>
         </is>
       </c>
       <c r="F42" s="13" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
+          <t>Grupp 4</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Blå</t>
+          <t>Alingsås HK Vit</t>
         </is>
       </c>
       <c r="I42" s="14" t="inlineStr">
         <is>
-          <t>Malmslätts HF</t>
+          <t>Lödde Vikings HK Röd</t>
         </is>
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>Malmslätts HF</t>
+          <t>Lödde Vikings HK Röd</t>
         </is>
       </c>
       <c r="K42" s="13" t="inlineStr">
@@ -2692,11 +2692,11 @@
         </is>
       </c>
       <c r="D43" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="E43" s="10" t="inlineStr">
-        <is>
-          <t>P15 Vit</t>
+        <v>16</v>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>P15 Blå</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr">
@@ -2706,22 +2706,22 @@
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
+          <t>Grupp 2</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK VIT</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="I43" s="14" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 3</t>
+          <t>Malmslätts HF</t>
         </is>
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 3</t>
+          <t>Malmslätts HF</t>
         </is>
       </c>
       <c r="K43" s="13" t="inlineStr">
@@ -2743,15 +2743,15 @@
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="D44" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="E44" s="11" t="inlineStr">
-        <is>
-          <t>P15 Orange</t>
+        <v>8</v>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>P15 Vit</t>
         </is>
       </c>
       <c r="F44" s="13" t="inlineStr">
@@ -2761,27 +2761,27 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
-        </is>
-      </c>
-      <c r="H44" s="14" t="inlineStr">
-        <is>
-          <t>Dalby GIF 1</t>
-        </is>
-      </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Orange</t>
+          <t>Grupp 1</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK VIT</t>
+        </is>
+      </c>
+      <c r="I44" s="14" t="inlineStr">
+        <is>
+          <t>IFK Kristianstad 3</t>
         </is>
       </c>
       <c r="J44" s="14" t="inlineStr">
         <is>
-          <t>Dalby GIF 1</t>
+          <t>IFK Kristianstad 3</t>
         </is>
       </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -2798,20 +2798,20 @@
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D45" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>F15 Vit</t>
+        <v>8</v>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>P15 Orange</t>
         </is>
       </c>
       <c r="F45" s="13" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="G45" s="13" t="inlineStr">
@@ -2819,24 +2819,24 @@
           <t>Grupp 4</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Vit</t>
-        </is>
-      </c>
-      <c r="I45" s="14" t="inlineStr">
-        <is>
-          <t>Ystads IF HF 1</t>
+      <c r="H45" s="14" t="inlineStr">
+        <is>
+          <t>IFK Malmö HF 2</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Orange</t>
         </is>
       </c>
       <c r="J45" s="14" t="inlineStr">
         <is>
-          <t>Ystads IF HF 1</t>
+          <t>IFK Malmö HF 2</t>
         </is>
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -2857,11 +2857,11 @@
         </is>
       </c>
       <c r="D46" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>F15 Blå</t>
+        <v>13</v>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>F15 Vit</t>
         </is>
       </c>
       <c r="F46" s="13" t="inlineStr">
@@ -2871,27 +2871,27 @@
       </c>
       <c r="G46" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
-        </is>
-      </c>
-      <c r="H46" s="14" t="inlineStr">
-        <is>
-          <t>Lödde Vikings HK Svart</t>
-        </is>
-      </c>
-      <c r="I46" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Blå</t>
+          <t>Grupp 4</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Vit</t>
+        </is>
+      </c>
+      <c r="I46" s="14" t="inlineStr">
+        <is>
+          <t>Ystads IF HF 1</t>
         </is>
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>Lödde Vikings HK Svart</t>
+          <t>Ystads IF HF 1</t>
         </is>
       </c>
       <c r="K46" s="13" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -2912,11 +2912,11 @@
         </is>
       </c>
       <c r="D47" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>F15 Gul</t>
+        <v>2</v>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>F15 Blå</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr">
@@ -2926,22 +2926,22 @@
       </c>
       <c r="G47" s="13" t="inlineStr">
         <is>
-          <t>Grupp 3</t>
+          <t>Grupp 1</t>
         </is>
       </c>
       <c r="H47" s="14" t="inlineStr">
         <is>
-          <t>Önnereds HK 1</t>
+          <t>Lödde Vikings HK Svart</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Gul</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="J47" s="14" t="inlineStr">
         <is>
-          <t>Önnereds HK 1</t>
+          <t>Lödde Vikings HK Svart</t>
         </is>
       </c>
       <c r="K47" s="13" t="inlineStr">
@@ -2963,40 +2963,40 @@
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="D48" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="E48" s="9" t="inlineStr">
-        <is>
-          <t>P15 Blå</t>
+        <v>8</v>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>F15 Gul</t>
         </is>
       </c>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="G48" s="13" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
+          <t>Grupp 3</t>
         </is>
       </c>
       <c r="H48" s="14" t="inlineStr">
         <is>
-          <t>HF Karlskrona Svart</t>
+          <t>Önnereds HK 1</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Blå</t>
+          <t>Alingsås HK Gul</t>
         </is>
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>HF Karlskrona Svart</t>
+          <t>Önnereds HK 1</t>
         </is>
       </c>
       <c r="K48" s="13" t="inlineStr">
@@ -3022,11 +3022,11 @@
         </is>
       </c>
       <c r="D49" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="E49" s="10" t="inlineStr">
-        <is>
-          <t>P15 Vit</t>
+        <v>15</v>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>P15 Blå</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr">
@@ -3036,22 +3036,22 @@
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
+          <t>Grupp 2</t>
         </is>
       </c>
       <c r="H49" s="14" t="inlineStr">
         <is>
-          <t>H43 Lund HF 1</t>
+          <t>HF Karlskrona Svart</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK VIT</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="J49" s="14" t="inlineStr">
         <is>
-          <t>H43 Lund HF 1</t>
+          <t>HF Karlskrona Svart</t>
         </is>
       </c>
       <c r="K49" s="13" t="inlineStr">
@@ -3073,15 +3073,15 @@
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="D50" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="E50" s="11" t="inlineStr">
-        <is>
-          <t>P15 Orange</t>
+        <v>8</v>
+      </c>
+      <c r="E50" s="10" t="inlineStr">
+        <is>
+          <t>P15 Vit</t>
         </is>
       </c>
       <c r="F50" s="13" t="inlineStr">
@@ -3091,22 +3091,22 @@
       </c>
       <c r="G50" s="13" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
+          <t>Grupp 1</t>
         </is>
       </c>
       <c r="H50" s="14" t="inlineStr">
         <is>
-          <t>IF Hallby HK Svart</t>
+          <t>H43 Lund HF 1</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Orange</t>
+          <t>Alingsås HK VIT</t>
         </is>
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>IF Hallby HK Svart</t>
+          <t>H43 Lund HF 1</t>
         </is>
       </c>
       <c r="K50" s="13" t="inlineStr">
@@ -3128,45 +3128,45 @@
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D51" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="E51" s="12" t="inlineStr">
-        <is>
-          <t>F15 Gul</t>
+        <v>12</v>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>P15 Orange</t>
         </is>
       </c>
       <c r="F51" s="13" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>P15</t>
         </is>
       </c>
       <c r="G51" s="13" t="inlineStr">
         <is>
-          <t>Grupp 3</t>
-        </is>
-      </c>
-      <c r="H51" s="14" t="inlineStr">
-        <is>
-          <t>IFK Tumba HK Vit</t>
-        </is>
-      </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Gul</t>
+          <t>Grupp 4</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Orange</t>
+        </is>
+      </c>
+      <c r="I51" s="14" t="inlineStr">
+        <is>
+          <t>Lödde Vikings HK</t>
         </is>
       </c>
       <c r="J51" s="14" t="inlineStr">
         <is>
-          <t>IFK Tumba HK Vit</t>
+          <t>Lödde Vikings HK</t>
         </is>
       </c>
       <c r="K51" s="13" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -3187,11 +3187,11 @@
         </is>
       </c>
       <c r="D52" s="13" t="n">
-        <v>17</v>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>F15 Vit</t>
+        <v>13</v>
+      </c>
+      <c r="E52" s="12" t="inlineStr">
+        <is>
+          <t>F15 Gul</t>
         </is>
       </c>
       <c r="F52" s="13" t="inlineStr">
@@ -3201,27 +3201,27 @@
       </c>
       <c r="G52" s="13" t="inlineStr">
         <is>
-          <t>Grupp 4</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Vit</t>
-        </is>
-      </c>
-      <c r="I52" s="14" t="inlineStr">
-        <is>
-          <t>Huddinge HK 2</t>
+          <t>Grupp 3</t>
+        </is>
+      </c>
+      <c r="H52" s="14" t="inlineStr">
+        <is>
+          <t>IFK Tumba HK Vit</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Gul</t>
         </is>
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>Huddinge HK 2</t>
+          <t>IFK Tumba HK Vit</t>
         </is>
       </c>
       <c r="K52" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -3242,11 +3242,11 @@
         </is>
       </c>
       <c r="D53" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>F15 Blå</t>
+        <v>17</v>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>F15 Vit</t>
         </is>
       </c>
       <c r="F53" s="13" t="inlineStr">
@@ -3256,22 +3256,22 @@
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>Grupp 1</t>
+          <t>Grupp 4</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK Blå</t>
+          <t>Alingsås HK Vit</t>
         </is>
       </c>
       <c r="I53" s="14" t="inlineStr">
         <is>
-          <t>Huddinge HK 1</t>
+          <t>Huddinge HK 2</t>
         </is>
       </c>
       <c r="J53" s="14" t="inlineStr">
         <is>
-          <t>Huddinge HK 1</t>
+          <t>Huddinge HK 2</t>
         </is>
       </c>
       <c r="K53" s="13" t="inlineStr">
@@ -3293,20 +3293,20 @@
       </c>
       <c r="C54" s="13" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D54" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="E54" s="10" t="inlineStr">
-        <is>
-          <t>P15 Vit</t>
+        <v>3</v>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>F15 Blå</t>
         </is>
       </c>
       <c r="F54" s="13" t="inlineStr">
         <is>
-          <t>P15</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="G54" s="13" t="inlineStr">
@@ -3316,17 +3316,17 @@
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>Alingsås HK VIT</t>
+          <t>Alingsås HK Blå</t>
         </is>
       </c>
       <c r="I54" s="14" t="inlineStr">
         <is>
-          <t>HF Karlskrona Blå</t>
+          <t>Huddinge HK 1</t>
         </is>
       </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>HF Karlskrona Blå</t>
+          <t>Huddinge HK 1</t>
         </is>
       </c>
       <c r="K54" s="13" t="inlineStr">
@@ -3348,15 +3348,15 @@
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="D55" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="9" t="inlineStr">
-        <is>
-          <t>P15 Blå</t>
+        <v>13</v>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
+        <is>
+          <t>P15 Vit</t>
         </is>
       </c>
       <c r="F55" s="13" t="inlineStr">
@@ -3366,27 +3366,27 @@
       </c>
       <c r="G55" s="13" t="inlineStr">
         <is>
-          <t>Grupp 2</t>
-        </is>
-      </c>
-      <c r="H55" s="14" t="inlineStr">
-        <is>
-          <t>IFK Kristianstad 2</t>
-        </is>
-      </c>
-      <c r="I55" s="6" t="inlineStr">
-        <is>
-          <t>Alingsås HK Blå</t>
+          <t>Grupp 1</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK VIT</t>
+        </is>
+      </c>
+      <c r="I55" s="14" t="inlineStr">
+        <is>
+          <t>HF Karlskrona Blå</t>
         </is>
       </c>
       <c r="J55" s="14" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 2</t>
+          <t>HF Karlskrona Blå</t>
         </is>
       </c>
       <c r="K55" s="13" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -3407,46 +3407,101 @@
         </is>
       </c>
       <c r="D56" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="E56" s="11" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>P15 Blå</t>
+        </is>
+      </c>
+      <c r="F56" s="13" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="G56" s="13" t="inlineStr">
+        <is>
+          <t>Grupp 2</t>
+        </is>
+      </c>
+      <c r="H56" s="14" t="inlineStr">
+        <is>
+          <t>IFK Kristianstad 2</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Blå</t>
+        </is>
+      </c>
+      <c r="J56" s="14" t="inlineStr">
+        <is>
+          <t>IFK Kristianstad 2</t>
+        </is>
+      </c>
+      <c r="K56" s="13" t="inlineStr">
+        <is>
+          <t>Borta</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>18/7</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>Lördag</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
         <is>
           <t>P15 Orange</t>
         </is>
       </c>
-      <c r="F56" s="13" t="inlineStr">
+      <c r="F57" s="13" t="inlineStr">
         <is>
           <t>P15</t>
         </is>
       </c>
-      <c r="G56" s="13" t="inlineStr">
+      <c r="G57" s="13" t="inlineStr">
         <is>
           <t>Grupp 4</t>
         </is>
       </c>
-      <c r="H56" s="14" t="inlineStr">
-        <is>
-          <t>Lödde Vikings HK</t>
-        </is>
-      </c>
-      <c r="I56" s="6" t="inlineStr">
+      <c r="H57" s="14" t="inlineStr">
+        <is>
+          <t>IFK Kristianstad 1</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
         <is>
           <t>Alingsås HK Orange</t>
         </is>
       </c>
-      <c r="J56" s="14" t="inlineStr">
-        <is>
-          <t>Lödde Vikings HK</t>
-        </is>
-      </c>
-      <c r="K56" s="13" t="inlineStr">
+      <c r="J57" s="14" t="inlineStr">
+        <is>
+          <t>IFK Kristianstad 1</t>
+        </is>
+      </c>
+      <c r="K57" s="13" t="inlineStr">
         <is>
           <t>Borta</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:K56"/>
+  <autoFilter ref="A5:K57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4052,7 +4107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4175,7 +4230,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 1</t>
+          <t>Spånga HK Vit</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -4185,7 +4240,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>IFK Kristianstad 1</t>
+          <t>Spånga HK Vit</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -4211,7 +4266,7 @@
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
@@ -4266,7 +4321,7 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
@@ -4283,24 +4338,24 @@
           <t>Grupp 4</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Eslövs HK Svart</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Alingsås HK Orange</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>Spånga HK Vit</t>
-        </is>
-      </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Spånga HK Vit</t>
+          <t>Eslövs HK Svart</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -4338,24 +4393,24 @@
           <t>Grupp 4</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>Eslövs HK Svart</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Alingsås HK Orange</t>
         </is>
       </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Lugi HF 4</t>
+        </is>
+      </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>Eslövs HK Svart</t>
+          <t>Lugi HF 4</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Borta</t>
+          <t>Hemma</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4431,7 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
@@ -4400,12 +4455,12 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Lugi HF 4</t>
+          <t>Täby HBK</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Lugi HF 4</t>
+          <t>Täby HBK</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -4427,11 +4482,11 @@
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D10" s="13" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
@@ -4448,24 +4503,24 @@
           <t>Grupp 4</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>Dalby GIF 1</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Alingsås HK Orange</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr">
-        <is>
-          <t>Täby HBK</t>
-        </is>
-      </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>Täby HBK</t>
+          <t>Dalby GIF 1</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>Hemma</t>
+          <t>Borta</t>
         </is>
       </c>
     </row>
@@ -4482,11 +4537,11 @@
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
@@ -4505,7 +4560,7 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>Dalby GIF 1</t>
+          <t>IF Hallby HK Svart</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -4515,7 +4570,7 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>Dalby GIF 1</t>
+          <t>IF Hallby HK Svart</t>
         </is>
       </c>
       <c r="K11" s="13" t="inlineStr">
@@ -4537,11 +4592,11 @@
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
@@ -4560,7 +4615,7 @@
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>IF Hallby HK Svart</t>
+          <t>IFK Malmö HF 2</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -4570,7 +4625,7 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>IF Hallby HK Svart</t>
+          <t>IFK Malmö HF 2</t>
         </is>
       </c>
       <c r="K12" s="13" t="inlineStr">
@@ -4592,7 +4647,7 @@
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="D13" s="13" t="n">
@@ -4613,22 +4668,77 @@
           <t>Grupp 4</t>
         </is>
       </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Alingsås HK Orange</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
         <is>
           <t>Lödde Vikings HK</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>Lödde Vikings HK</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>Hemma</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>18/7</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Lördag</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>P15 Orange</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>P15</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>Grupp 4</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>IFK Kristianstad 1</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Alingsås HK Orange</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>Lödde Vikings HK</t>
-        </is>
-      </c>
-      <c r="K13" s="13" t="inlineStr">
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>IFK Kristianstad 1</t>
+        </is>
+      </c>
+      <c r="K14" s="13" t="inlineStr">
         <is>
           <t>Borta</t>
         </is>
@@ -4774,12 +4884,12 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>IFK Malmö HF</t>
+          <t>IFK Malmö HF 1</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>IFK Malmö HF</t>
+          <t>IFK Malmö HF 1</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">

</xml_diff>